<commit_message>
📊 Update: tlak_data.json z Excel (21 měření) + database schema diagram
</commit_message>
<xml_diff>
--- a/Krevni_tlak_Pavel.xlsx
+++ b/Krevni_tlak_Pavel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pavel.hlousek/Documents/Claude/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF7D49E-910E-8142-8025-3A3086FD703A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E5913D0-E6AC-C64D-B699-2086398D7E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="24100" windowHeight="15380" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="156">
   <si>
     <t>Deník krevního tlaku  ·  Pavel</t>
   </si>
@@ -505,6 +505,12 @@
   </si>
   <si>
     <t>ráno divně v puse - lék Controloc si nevezmu, ale ranní Meditace Dispensa, večer stažený krk jako včera</t>
+  </si>
+  <si>
+    <t>pořád cítím bolest v krku v oblasti hlasivek</t>
+  </si>
+  <si>
+    <t>a odjíždím do HK a Anglie - bez sledování tlaku</t>
   </si>
 </sst>
 </file>
@@ -1119,19 +1125,19 @@
                   <c:v>118.5</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>117</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
+                  <c:v>105</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0</c:v>
+                  <c:v>118</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>0</c:v>
@@ -1466,19 +1472,19 @@
                   <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>77.5</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0</c:v>
+                  <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>0</c:v>
@@ -2090,19 +2096,19 @@
                   <c:v>123</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>109.5</c:v>
                 </c:pt>
                 <c:pt idx="18">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
+                  <c:v>118</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0</c:v>
@@ -2437,19 +2443,19 @@
                   <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>72</c:v>
                 </c:pt>
                 <c:pt idx="18">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0</c:v>
+                  <c:v>77.5</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
+                  <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>71.5</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0</c:v>
@@ -4523,55 +4529,81 @@
         <f t="shared" si="3"/>
         <v>Normální</v>
       </c>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
-      <c r="N22" s="12"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="10" t="str">
+      <c r="L22" s="13">
+        <v>106</v>
+      </c>
+      <c r="M22" s="13">
+        <v>75</v>
+      </c>
+      <c r="N22" s="13">
+        <v>58</v>
+      </c>
+      <c r="O22" s="12">
+        <v>113</v>
+      </c>
+      <c r="P22" s="12">
+        <v>69</v>
+      </c>
+      <c r="Q22" s="12">
+        <v>57</v>
+      </c>
+      <c r="R22" s="10">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="S22" s="10" t="str">
+        <v>109.5</v>
+      </c>
+      <c r="S22" s="10">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="T22" s="10" t="str">
+        <v>72</v>
+      </c>
+      <c r="T22" s="10">
         <f t="shared" si="6"/>
-        <v/>
+        <v>57.5</v>
       </c>
       <c r="U22" s="11" t="str">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="V22" s="16"/>
+        <v>Normální</v>
+      </c>
+      <c r="V22" s="16" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="23" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="10" t="str">
+      <c r="B23" s="8">
+        <v>119</v>
+      </c>
+      <c r="C23" s="8">
+        <v>79</v>
+      </c>
+      <c r="D23" s="8">
+        <v>55</v>
+      </c>
+      <c r="E23" s="9">
+        <v>115</v>
+      </c>
+      <c r="F23" s="9">
+        <v>76</v>
+      </c>
+      <c r="G23" s="9">
+        <v>55</v>
+      </c>
+      <c r="H23" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I23" s="10" t="str">
+        <v>117</v>
+      </c>
+      <c r="I23" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J23" s="10" t="str">
+        <v>77.5</v>
+      </c>
+      <c r="J23" s="10">
         <f t="shared" si="2"/>
-        <v/>
+        <v>55</v>
       </c>
       <c r="K23" s="11" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Normální</v>
       </c>
       <c r="L23" s="12"/>
       <c r="M23" s="12"/>
@@ -4623,27 +4655,39 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L24" s="12"/>
-      <c r="M24" s="12"/>
-      <c r="N24" s="12"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="13"/>
-      <c r="R24" s="10" t="str">
+      <c r="L24" s="12">
+        <v>128</v>
+      </c>
+      <c r="M24" s="12">
+        <v>81</v>
+      </c>
+      <c r="N24" s="12">
+        <v>53</v>
+      </c>
+      <c r="O24" s="13">
+        <v>112</v>
+      </c>
+      <c r="P24" s="13">
+        <v>74</v>
+      </c>
+      <c r="Q24" s="13">
+        <v>53</v>
+      </c>
+      <c r="R24" s="10">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="S24" s="10" t="str">
+        <v>120</v>
+      </c>
+      <c r="S24" s="10">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="T24" s="10" t="str">
+        <v>77.5</v>
+      </c>
+      <c r="T24" s="10">
         <f t="shared" si="6"/>
-        <v/>
+        <v>53</v>
       </c>
       <c r="U24" s="11" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>Normální</v>
       </c>
       <c r="V24" s="16"/>
     </row>
@@ -4651,49 +4695,67 @@
       <c r="A25" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
+      <c r="B25" s="8">
+        <v>105</v>
+      </c>
+      <c r="C25" s="8">
+        <v>74</v>
+      </c>
+      <c r="D25" s="8">
+        <v>54</v>
+      </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
-      <c r="H25" s="10" t="str">
+      <c r="H25" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I25" s="10" t="str">
+        <v>105</v>
+      </c>
+      <c r="I25" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J25" s="10" t="str">
+        <v>74</v>
+      </c>
+      <c r="J25" s="10">
         <f t="shared" si="2"/>
-        <v/>
+        <v>54</v>
       </c>
       <c r="K25" s="11" t="str">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L25" s="12"/>
-      <c r="M25" s="12"/>
-      <c r="N25" s="12"/>
-      <c r="O25" s="13"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="13"/>
-      <c r="R25" s="10" t="str">
+        <v>Normální</v>
+      </c>
+      <c r="L25" s="12">
+        <v>118</v>
+      </c>
+      <c r="M25" s="12">
+        <v>75</v>
+      </c>
+      <c r="N25" s="12">
+        <v>59</v>
+      </c>
+      <c r="O25" s="13">
+        <v>118</v>
+      </c>
+      <c r="P25" s="13">
+        <v>79</v>
+      </c>
+      <c r="Q25" s="13">
+        <v>60</v>
+      </c>
+      <c r="R25" s="10">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="S25" s="10" t="str">
+        <v>118</v>
+      </c>
+      <c r="S25" s="10">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="T25" s="10" t="str">
+        <v>77</v>
+      </c>
+      <c r="T25" s="10">
         <f t="shared" si="6"/>
-        <v/>
+        <v>59.5</v>
       </c>
       <c r="U25" s="11" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>Normální</v>
       </c>
       <c r="V25" s="14"/>
     </row>
@@ -4701,49 +4763,73 @@
       <c r="A26" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="10" t="str">
+      <c r="B26" s="8">
+        <v>115</v>
+      </c>
+      <c r="C26" s="8">
+        <v>78</v>
+      </c>
+      <c r="D26" s="8">
+        <v>52</v>
+      </c>
+      <c r="E26" s="9">
+        <v>115</v>
+      </c>
+      <c r="F26" s="9">
+        <v>76</v>
+      </c>
+      <c r="G26" s="9">
+        <v>51</v>
+      </c>
+      <c r="H26" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I26" s="10" t="str">
+        <v>115</v>
+      </c>
+      <c r="I26" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J26" s="10" t="str">
+        <v>77</v>
+      </c>
+      <c r="J26" s="10">
         <f t="shared" si="2"/>
-        <v/>
+        <v>51.5</v>
       </c>
       <c r="K26" s="11" t="str">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="10" t="str">
+        <v>Normální</v>
+      </c>
+      <c r="L26" s="12">
+        <v>112</v>
+      </c>
+      <c r="M26" s="12">
+        <v>71</v>
+      </c>
+      <c r="N26" s="12">
+        <v>65</v>
+      </c>
+      <c r="O26" s="13">
+        <v>108</v>
+      </c>
+      <c r="P26" s="13">
+        <v>72</v>
+      </c>
+      <c r="Q26" s="13">
+        <v>67</v>
+      </c>
+      <c r="R26" s="10">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="S26" s="10" t="str">
+        <v>110</v>
+      </c>
+      <c r="S26" s="10">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="T26" s="10" t="str">
+        <v>71.5</v>
+      </c>
+      <c r="T26" s="10">
         <f t="shared" si="6"/>
-        <v/>
+        <v>66</v>
       </c>
       <c r="U26" s="11" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>Normální</v>
       </c>
       <c r="V26" s="16"/>
     </row>
@@ -4751,27 +4837,39 @@
       <c r="A27" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="10" t="str">
+      <c r="B27" s="8">
+        <v>115</v>
+      </c>
+      <c r="C27" s="8">
+        <v>76</v>
+      </c>
+      <c r="D27" s="8">
+        <v>61</v>
+      </c>
+      <c r="E27" s="9">
+        <v>121</v>
+      </c>
+      <c r="F27" s="9">
+        <v>78</v>
+      </c>
+      <c r="G27" s="9">
+        <v>63</v>
+      </c>
+      <c r="H27" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I27" s="10" t="str">
+        <v>118</v>
+      </c>
+      <c r="I27" s="10">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J27" s="10" t="str">
+        <v>77</v>
+      </c>
+      <c r="J27" s="10">
         <f t="shared" si="2"/>
-        <v/>
+        <v>62</v>
       </c>
       <c r="K27" s="11" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Normální</v>
       </c>
       <c r="L27" s="12"/>
       <c r="M27" s="12"/>
@@ -4795,7 +4893,9 @@
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="V27" s="14"/>
+      <c r="V27" s="14" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="28" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="15" t="s">
@@ -8219,15 +8319,15 @@
       </c>
       <c r="B5" s="19">
         <f>IFERROR(AVERAGEIF('Denní log'!H5:H94,"&lt;&gt;",'Denní log'!H5:H94),"-")</f>
-        <v>123.23333333333333</v>
+        <v>121.23684210526316</v>
       </c>
       <c r="C5" s="19">
         <f>IFERROR(AVERAGEIF('Denní log'!I5:I94,"&lt;&gt;",'Denní log'!I5:I94),"-")</f>
-        <v>77.933333333333337</v>
+        <v>77.60526315789474</v>
       </c>
       <c r="D5" s="19">
         <f>IFERROR(AVERAGEIF('Denní log'!J5:J94,"&lt;&gt;",'Denní log'!J5:J94),"-")</f>
-        <v>55.733333333333334</v>
+        <v>55.710526315789473</v>
       </c>
       <c r="E5" s="20">
         <f>COUNTIF('Denní log'!H5:H94,"&lt;&gt;"&amp;"")</f>
@@ -8276,15 +8376,15 @@
       </c>
       <c r="B8" s="19">
         <f>IFERROR(LOOKUP(2,1/('Denní log'!H5:H94&lt;&gt;""),'Denní log'!H5:H94),"-")</f>
-        <v>118.5</v>
+        <v>118</v>
       </c>
       <c r="C8" s="19">
         <f>IFERROR(LOOKUP(2,1/('Denní log'!I5:I94&lt;&gt;""),'Denní log'!I5:I94),"-")</f>
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D8" s="19">
         <f>IFERROR(LOOKUP(2,1/('Denní log'!J5:J94&lt;&gt;""),'Denní log'!J5:J94),"-")</f>
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="E8" s="20"/>
     </row>
@@ -8321,15 +8421,15 @@
       </c>
       <c r="B12" s="19">
         <f>IFERROR(AVERAGEIF('Denní log'!R5:R94,"&lt;&gt;",'Denní log'!R5:R94),"-")</f>
-        <v>124.75</v>
+        <v>122.44444444444444</v>
       </c>
       <c r="C12" s="19">
         <f>IFERROR(AVERAGEIF('Denní log'!S5:S94,"&lt;&gt;",'Denní log'!S5:S94),"-")</f>
-        <v>75.214285714285708</v>
+        <v>75.055555555555557</v>
       </c>
       <c r="D12" s="19">
         <f>IFERROR(AVERAGEIF('Denní log'!T5:T94,"&lt;&gt;",'Denní log'!T5:T94),"-")</f>
-        <v>56.642857142857146</v>
+        <v>57.166666666666664</v>
       </c>
       <c r="E12" s="20">
         <f>COUNTIF('Denní log'!R5:R94,"&lt;&gt;"&amp;"")</f>
@@ -8378,15 +8478,15 @@
       </c>
       <c r="B15" s="19">
         <f>IFERROR(LOOKUP(2,1/('Denní log'!R5:R94&lt;&gt;""),'Denní log'!R5:R94),"-")</f>
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C15" s="19">
         <f>IFERROR(LOOKUP(2,1/('Denní log'!S5:S94&lt;&gt;""),'Denní log'!S5:S94),"-")</f>
-        <v>75</v>
+        <v>71.5</v>
       </c>
       <c r="D15" s="19">
         <f>IFERROR(LOOKUP(2,1/('Denní log'!T5:T94&lt;&gt;""),'Denní log'!T5:T94),"-")</f>
-        <v>62.5</v>
+        <v>66</v>
       </c>
       <c r="E15" s="20"/>
     </row>

</xml_diff>